<commit_message>
Fix GMV parsing (month-labelled headers); overwrite-merge both sheets, blank+email on conflict
</commit_message>
<xml_diff>
--- a/snapshots/mkt_snapshot.xlsx
+++ b/snapshots/mkt_snapshot.xlsx
@@ -2276,12 +2276,24 @@
       <c r="J22" t="n">
         <v>126866.73</v>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
+      <c r="K22" t="n">
+        <v>180</v>
+      </c>
+      <c r="L22" t="n">
+        <v>241684</v>
+      </c>
+      <c r="M22" t="n">
+        <v>185709</v>
+      </c>
+      <c r="N22" t="n">
+        <v>205</v>
+      </c>
+      <c r="O22" t="n">
+        <v>245499</v>
+      </c>
+      <c r="P22" t="n">
+        <v>282791</v>
+      </c>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
@@ -2341,12 +2353,24 @@
       <c r="J23" t="n">
         <v>125305.89</v>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
+      <c r="K23" t="n">
+        <v>227</v>
+      </c>
+      <c r="L23" t="n">
+        <v>301973</v>
+      </c>
+      <c r="M23" t="n">
+        <v>156406</v>
+      </c>
+      <c r="N23" t="n">
+        <v>248</v>
+      </c>
+      <c r="O23" t="n">
+        <v>280214</v>
+      </c>
+      <c r="P23" t="n">
+        <v>333204</v>
+      </c>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
@@ -2406,12 +2430,24 @@
       <c r="J24" t="n">
         <v>75734.33</v>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
+      <c r="K24" t="n">
+        <v>179</v>
+      </c>
+      <c r="L24" t="n">
+        <v>211755</v>
+      </c>
+      <c r="M24" t="n">
+        <v>148967</v>
+      </c>
+      <c r="N24" t="n">
+        <v>263</v>
+      </c>
+      <c r="O24" t="n">
+        <v>290691</v>
+      </c>
+      <c r="P24" t="n">
+        <v>276298</v>
+      </c>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
@@ -2471,12 +2507,24 @@
       <c r="J25" t="n">
         <v>108754.3</v>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
+      <c r="K25" t="n">
+        <v>179</v>
+      </c>
+      <c r="L25" t="n">
+        <v>230832</v>
+      </c>
+      <c r="M25" t="n">
+        <v>172007</v>
+      </c>
+      <c r="N25" t="n">
+        <v>286</v>
+      </c>
+      <c r="O25" t="n">
+        <v>293352</v>
+      </c>
+      <c r="P25" t="n">
+        <v>323498</v>
+      </c>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
@@ -2536,12 +2584,24 @@
       <c r="J26" t="n">
         <v>32875.25</v>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
+      <c r="K26" t="n">
+        <v>132</v>
+      </c>
+      <c r="L26" t="n">
+        <v>167691</v>
+      </c>
+      <c r="M26" t="n">
+        <v>171436</v>
+      </c>
+      <c r="N26" t="n">
+        <v>247</v>
+      </c>
+      <c r="O26" t="n">
+        <v>273597</v>
+      </c>
+      <c r="P26" t="n">
+        <v>331583</v>
+      </c>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
@@ -2601,12 +2661,24 @@
       <c r="J27" t="n">
         <v>70850.44</v>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
+      <c r="K27" t="n">
+        <v>133</v>
+      </c>
+      <c r="L27" t="n">
+        <v>176129</v>
+      </c>
+      <c r="M27" t="n">
+        <v>129972</v>
+      </c>
+      <c r="N27" t="n">
+        <v>339</v>
+      </c>
+      <c r="O27" t="n">
+        <v>369336</v>
+      </c>
+      <c r="P27" t="n">
+        <v>354744</v>
+      </c>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
@@ -2654,16 +2726,36 @@
       <c r="F28" t="n">
         <v>127998</v>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
+      <c r="G28" t="n">
+        <v>533</v>
+      </c>
+      <c r="H28" t="n">
+        <v>613669</v>
+      </c>
+      <c r="I28" t="n">
+        <v>433966</v>
+      </c>
+      <c r="J28" t="n">
+        <v>121805.71</v>
+      </c>
+      <c r="K28" t="n">
+        <v>130</v>
+      </c>
+      <c r="L28" t="n">
+        <v>166479</v>
+      </c>
+      <c r="M28" t="n">
+        <v>123303</v>
+      </c>
+      <c r="N28" t="n">
+        <v>398</v>
+      </c>
+      <c r="O28" t="n">
+        <v>438337</v>
+      </c>
+      <c r="P28" t="n">
+        <v>283140</v>
+      </c>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
@@ -2677,24 +2769,34 @@
       <c r="AA28" t="inlineStr"/>
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="n">
-        <v>88</v>
+        <v>621</v>
       </c>
       <c r="AD28" t="n">
-        <v>133334</v>
+        <v>747003</v>
       </c>
       <c r="AE28" t="n">
-        <v>70556</v>
+        <v>504522</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
+      <c r="B29" t="n">
+        <v>53</v>
+      </c>
+      <c r="C29" t="n">
+        <v>73912</v>
+      </c>
+      <c r="D29" t="n">
+        <v>153078</v>
+      </c>
+      <c r="E29" t="n">
+        <v>6</v>
+      </c>
+      <c r="F29" t="n">
+        <v>70837</v>
+      </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
@@ -2718,13 +2820,13 @@
       <c r="AA29" t="inlineStr"/>
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="AD29" t="n">
-        <v>0</v>
+        <v>73912</v>
       </c>
       <c r="AE29" t="n">
-        <v>0</v>
+        <v>153078</v>
       </c>
     </row>
     <row r="30">
@@ -2933,49 +3035,49 @@
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>1989</v>
+        <v>2042</v>
       </c>
       <c r="C35" t="n">
-        <v>2650381</v>
+        <v>2724293</v>
       </c>
       <c r="D35" t="n">
-        <v>1855075</v>
+        <v>2008153</v>
       </c>
       <c r="E35" t="n">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="F35" t="n">
-        <v>2290173</v>
+        <v>2361010</v>
       </c>
       <c r="G35" t="n">
-        <v>12478</v>
+        <v>13011</v>
       </c>
       <c r="H35" t="n">
-        <v>14398882</v>
+        <v>15012551</v>
       </c>
       <c r="I35" t="n">
-        <v>11744027.76</v>
+        <v>12177993.76</v>
       </c>
       <c r="J35" t="n">
-        <v>3310625.48</v>
+        <v>3432431.19</v>
       </c>
       <c r="K35" t="n">
-        <v>3759</v>
+        <v>4919</v>
       </c>
       <c r="L35" t="n">
-        <v>4549118</v>
+        <v>6045661</v>
       </c>
       <c r="M35" t="n">
-        <v>2965965</v>
+        <v>4053765</v>
       </c>
       <c r="N35" t="n">
-        <v>5989</v>
+        <v>7975</v>
       </c>
       <c r="O35" t="n">
-        <v>6572344</v>
+        <v>8763370</v>
       </c>
       <c r="P35" t="n">
-        <v>5869869</v>
+        <v>8055127</v>
       </c>
       <c r="Q35" t="n">
         <v>0</v>
@@ -3014,38 +3116,38 @@
         <v>2057025</v>
       </c>
       <c r="AC35" t="n">
-        <v>24454</v>
+        <v>25040</v>
       </c>
       <c r="AD35" t="n">
-        <v>25069153</v>
+        <v>25756734</v>
       </c>
       <c r="AE35" t="n">
-        <v>17524040.18855</v>
+        <v>18111084.18855</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>0.4287190544856677</v>
+        <v>0.3566162538412163</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>0.2260599424877381</v>
+        <v>0.2327606086735259</v>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="n">
-        <v>0.5337733250392368</v>
+        <v>0.4913693813035536</v>
       </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="n">
-        <v>0.1196747320936805</v>
+        <v>0.08792449827296329</v>
       </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
@@ -3066,21 +3168,21 @@
       <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="inlineStr"/>
       <c r="AD36" t="n">
-        <v>0.4305578354231289</v>
+        <v>0.4221530711167286</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
-        <v>3912467.190476191</v>
+        <v>3248195.5</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>17854613.68</v>
+        <v>17899580.03846154</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -3095,7 +3197,7 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="n">
-        <v>96309.25</v>
+        <v>46228.44</v>
       </c>
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
@@ -3105,12 +3207,12 @@
       <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="inlineStr"/>
       <c r="AA38" t="n">
-        <v>12849210.66666667</v>
+        <v>8566140.444444444</v>
       </c>
       <c r="AB38" t="inlineStr"/>
       <c r="AC38" t="inlineStr"/>
       <c r="AD38" t="n">
-        <v>39621566.62924813</v>
+        <v>34669110.26501124</v>
       </c>
     </row>
     <row r="39">
@@ -3178,7 +3280,7 @@
       <c r="AB40" t="inlineStr"/>
       <c r="AC40" t="inlineStr"/>
       <c r="AD40" t="n">
-        <v>97778100.77924812</v>
+        <v>92825644.41501124</v>
       </c>
     </row>
     <row r="41">

</xml_diff>

<commit_message>
Fix: sub-channels (Amazon Core/NOW+Fresh) were double-counted in totals
Amazon Core and NOW+Fresh are a split of Amazon, not extra business - Amazon's own GMV already includes them. Section subtotal and grand total were summing every channel in the section, so Amazon's business was counted twice: once as Amazon, once again as Core + NOW+Fresh.

Fixed in transform.py: section totals, the grand total, and link_previous's per-month recompute now exclude cadence=sub before summing. qc.py layer B's section-identity sums updated to match. Sub-channels still get their own row (tagged of Amazon) and the contribution strip; the roll-up math (parent vs sum of parts) is unaffected since it reads from summaries, not totals.

July 2026 (31 Jul, full month) grand GMV is now 8.78 Cr, down from the double-counted ~10.0 Cr. 518/518 checks pass; the 9-case negative test still catches every injected regression.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/snapshots/mkt_snapshot.xlsx
+++ b/snapshots/mkt_snapshot.xlsx
@@ -2880,9 +2880,15 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
+      <c r="T29" t="n">
+        <v>2</v>
+      </c>
+      <c r="U29" t="n">
+        <v>1441</v>
+      </c>
+      <c r="V29" t="n">
+        <v>1858</v>
+      </c>
       <c r="W29" t="n">
         <v>1864</v>
       </c>
@@ -2902,13 +2908,13 @@
         <v>297136</v>
       </c>
       <c r="AC29" t="n">
-        <v>2507</v>
+        <v>2509</v>
       </c>
       <c r="AD29" t="n">
-        <v>2014185</v>
+        <v>2015626</v>
       </c>
       <c r="AE29" t="n">
-        <v>988375</v>
+        <v>990233</v>
       </c>
     </row>
     <row r="30">
@@ -2951,9 +2957,15 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
+      <c r="T30" t="n">
+        <v>1</v>
+      </c>
+      <c r="U30" t="n">
+        <v>594</v>
+      </c>
+      <c r="V30" t="n">
+        <v>2052</v>
+      </c>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
@@ -2961,13 +2973,13 @@
       <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="n">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="AD30" t="n">
-        <v>516992</v>
+        <v>517586</v>
       </c>
       <c r="AE30" t="n">
-        <v>577714</v>
+        <v>579766</v>
       </c>
     </row>
     <row r="31">
@@ -3010,9 +3022,15 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
+      <c r="T31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" t="n">
+        <v>1036</v>
+      </c>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
       <c r="Y31" t="inlineStr"/>
@@ -3026,7 +3044,7 @@
         <v>565165</v>
       </c>
       <c r="AE31" t="n">
-        <v>547796</v>
+        <v>548832</v>
       </c>
     </row>
     <row r="32">
@@ -3061,9 +3079,15 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
+      <c r="T32" t="n">
+        <v>1</v>
+      </c>
+      <c r="U32" t="n">
+        <v>1609</v>
+      </c>
+      <c r="V32" t="n">
+        <v>594</v>
+      </c>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
       <c r="Y32" t="inlineStr"/>
@@ -3071,13 +3095,13 @@
       <c r="AA32" t="inlineStr"/>
       <c r="AB32" t="inlineStr"/>
       <c r="AC32" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="AD32" t="n">
-        <v>93127</v>
+        <v>94736</v>
       </c>
       <c r="AE32" t="n">
-        <v>89783</v>
+        <v>90377</v>
       </c>
     </row>
     <row r="33">
@@ -3217,13 +3241,13 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="U35" t="n">
-        <v>37281</v>
+        <v>40925</v>
       </c>
       <c r="V35" t="n">
-        <v>44498</v>
+        <v>50038</v>
       </c>
       <c r="W35" t="n">
         <v>6963</v>
@@ -3244,13 +3268,13 @@
         <v>4030860</v>
       </c>
       <c r="AC35" t="n">
-        <v>31629</v>
+        <v>31633</v>
       </c>
       <c r="AD35" t="n">
-        <v>30847355</v>
+        <v>30850999</v>
       </c>
       <c r="AE35" t="n">
-        <v>22534577.76</v>
+        <v>22540117.76</v>
       </c>
     </row>
     <row r="36">
@@ -3296,7 +3320,7 @@
       <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="inlineStr"/>
       <c r="AD36" t="n">
-        <v>0.3688898602198614</v>
+        <v>0.3687150763137804</v>
       </c>
     </row>
     <row r="38">
@@ -3329,7 +3353,7 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="n">
-        <v>46228.44</v>
+        <v>50747</v>
       </c>
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
@@ -3344,7 +3368,7 @@
       <c r="AB38" t="inlineStr"/>
       <c r="AC38" t="inlineStr"/>
       <c r="AD38" t="n">
-        <v>45288074.68589842</v>
+        <v>45292593.24589842</v>
       </c>
     </row>
     <row r="39">
@@ -3414,7 +3438,7 @@
       <c r="AB40" t="inlineStr"/>
       <c r="AC40" t="inlineStr"/>
       <c r="AD40" t="n">
-        <v>103444608.8358984</v>
+        <v>103449127.3958984</v>
       </c>
     </row>
     <row r="41">

</xml_diff>